<commit_message>
Update TOEIC_Words_401-500_List.csv to place Japanese translation adjacent to English word
</commit_message>
<xml_diff>
--- a/TOEIC_Words_401-500_100Quiz.xlsx
+++ b/TOEIC_Words_401-500_100Quiz.xlsx
@@ -265,11 +265,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -280,11 +280,11 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -768,8 +768,8 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -803,12 +803,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>主な意味 (Meaning)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>品詞</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>主な意味 (Meaning)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
+          <t>引き起こす</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>引き起こす</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
+          <t>10年</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>10年</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -908,12 +908,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
+          <t>期限が切れる</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>期限が切れる</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -943,12 +943,12 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
+          <t>収入</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>収入</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
+          <t>早急な</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>早急な</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
+          <t>アンケート</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>アンケート</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
+          <t>習慣的に繰り返されること</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>習慣的に繰り返されること</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1083,12 +1083,12 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
+          <t>転勤する</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>転勤する</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
+          <t>複雑な</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>複雑な</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
+          <t>教育</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>教育</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
+          <t>出迎える</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>出迎える</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
+          <t>影響力</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>影響力</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
+          <t>不足</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>不足</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
+          <t>温暖な</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>温暖な</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -1328,12 +1328,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
+          <t>普通は</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
           <t>副詞</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>普通は</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
+          <t>身体の</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>身体の</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -1398,12 +1398,12 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
+          <t>礼儀正しい</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>礼儀正しい</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
+          <t>人口</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>人口</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
+          <t>注ぐ</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>注ぐ</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
+          <t>すぐの</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>すぐの</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
+          <t>会場</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>会場</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
+          <t>辞任する</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>辞任する</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -1608,12 +1608,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
+          <t>添付する</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>添付する</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
+          <t>取り消す</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>取り消す</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
+          <t>よくある</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>よくある</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -1713,12 +1713,12 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
+          <t>会話</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>会話</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
+          <t>経済的な</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>経済的な</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1783,12 +1783,12 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
+          <t>交換する</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>交換する</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
+          <t>専門家</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>専門家</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -1853,12 +1853,12 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
+          <t>内線</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>内線</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
+          <t>よく知っている</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>よく知っている</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -1923,12 +1923,12 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
+          <t>主催する</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t>主催する</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -1958,12 +1958,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
+          <t>車に乗せること</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>車に乗せること</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
+          <t>求める</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>求める</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -2028,12 +2028,12 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
+          <t>辞任する(身を引く)</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>辞任する(身を引く)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
+          <t>手法</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>手法</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
@@ -2098,12 +2098,12 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
+          <t>臨時の</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>臨時の</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2133,12 +2133,12 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
+          <t>要因</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
-        <is>
-          <t>要因</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -2168,12 +2168,12 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
+          <t>組み立てる</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>組み立てる</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
+          <t>注意</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D44" s="12" t="inlineStr">
-        <is>
-          <t>注意</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
+          <t>請求書</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>請求書</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -2273,12 +2273,12 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
+          <t>〜の前に</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
           <t>前置詞</t>
-        </is>
-      </c>
-      <c r="D46" s="12" t="inlineStr">
-        <is>
-          <t>〜の前に</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
+          <t>軽い飲食料</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>軽い飲食料</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2343,12 +2343,12 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
+          <t>信用</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t>信用</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -2378,12 +2378,12 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
+          <t>配管工</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>配管工</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -2413,12 +2413,12 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
+          <t>更新する</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D50" s="12" t="inlineStr">
-        <is>
-          <t>更新する</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -2448,12 +2448,12 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
+          <t>上の階に</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
           <t>副詞</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>上の階に</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -2483,12 +2483,12 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
+          <t>態度</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D52" s="12" t="inlineStr">
-        <is>
-          <t>態度</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
+          <t>考える</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>考える</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
+          <t>重役</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>重役</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -2588,12 +2588,12 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
+          <t>手段</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>手段</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -2623,12 +2623,12 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
+          <t>〜に関する</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
           <t>前置詞</t>
-        </is>
-      </c>
-      <c r="D56" s="12" t="inlineStr">
-        <is>
-          <t>〜に関する</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -2658,12 +2658,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
+          <t>提携</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>提携</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -2693,12 +2693,12 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
+          <t>予算</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D58" s="12" t="inlineStr">
-        <is>
-          <t>予算</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -2728,12 +2728,12 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
+          <t>含む</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>含む</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
+          <t>〜のままでいる</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>〜のままでいる</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
@@ -2798,12 +2798,12 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
+          <t>化学薬品</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>化学薬品</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -2833,12 +2833,12 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
+          <t>実地説明をする</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D62" s="12" t="inlineStr">
-        <is>
-          <t>実地説明をする</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -2868,12 +2868,12 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
+          <t>適任である</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>適任である</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -2903,12 +2903,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
+          <t>修正する</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>修正する</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -2938,12 +2938,12 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
+          <t>くつろいだ</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D65" s="7" t="inlineStr">
-        <is>
-          <t>くつろいだ</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -2973,12 +2973,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
+          <t>改良する</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D66" s="12" t="inlineStr">
-        <is>
-          <t>改良する</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -3008,12 +3008,12 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
+          <t>同行する</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>同行する</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -3043,12 +3043,12 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
+          <t>態度(姿勢)</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t>態度(姿勢)</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
@@ -3078,12 +3078,12 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
+          <t>通勤する</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>通勤する</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
+          <t>競争力のある</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D70" s="12" t="inlineStr">
-        <is>
-          <t>競争力のある</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -3148,12 +3148,12 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
+          <t>拒否する</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>拒否する</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -3183,12 +3183,12 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
+          <t>定期購読する</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D72" s="12" t="inlineStr">
-        <is>
-          <t>定期購読する</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -3218,12 +3218,12 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
+          <t>処理する</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>処理する</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -3253,12 +3253,12 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
+          <t>意見</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D74" s="12" t="inlineStr">
-        <is>
-          <t>意見</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
+          <t>必要な</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>必要な</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -3323,12 +3323,12 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
+          <t>それぞれ</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
           <t>副詞</t>
-        </is>
-      </c>
-      <c r="D76" s="12" t="inlineStr">
-        <is>
-          <t>それぞれ</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
+          <t>起こりそうな</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>起こりそうな</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
+          <t>効率のよい</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D78" s="12" t="inlineStr">
-        <is>
-          <t>効率のよい</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
@@ -3428,12 +3428,12 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
+          <t>明らかにする</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t>明らかにする</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
+          <t>特定の</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D80" s="12" t="inlineStr">
-        <is>
-          <t>特定の</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
@@ -3498,12 +3498,12 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
+          <t>移転する</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>移転する</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -3533,12 +3533,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
+          <t>思い出させる</t>
+        </is>
+      </c>
+      <c r="D82" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D82" s="12" t="inlineStr">
-        <is>
-          <t>思い出させる</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
@@ -3568,12 +3568,12 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
+          <t>〜と比べて</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
           <t>熟語</t>
-        </is>
-      </c>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t>〜と比べて</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -3603,12 +3603,12 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
+          <t>設立する</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D84" s="12" t="inlineStr">
-        <is>
-          <t>設立する</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
@@ -3638,12 +3638,12 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
+          <t>指摘する</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
           <t>句動詞</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>指摘する</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -3673,12 +3673,12 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
+          <t>不動産</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D86" s="12" t="inlineStr">
-        <is>
-          <t>不動産</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
@@ -3708,12 +3708,12 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
+          <t>修復する</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>修復する</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -3743,12 +3743,12 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
+          <t>状況</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D88" s="12" t="inlineStr">
-        <is>
-          <t>状況</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
@@ -3778,12 +3778,12 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
+          <t>経費</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>経費</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -3813,12 +3813,12 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
+          <t>焦点を合わせる</t>
+        </is>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D90" s="12" t="inlineStr">
-        <is>
-          <t>焦点を合わせる</t>
         </is>
       </c>
       <c r="E90" s="13" t="inlineStr">
@@ -3848,12 +3848,12 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
+          <t>研究所</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>研究所</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -3883,12 +3883,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
+          <t>得る</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D92" s="12" t="inlineStr">
-        <is>
-          <t>得る</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr">
@@ -3918,12 +3918,12 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
+          <t>評判</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D93" s="7" t="inlineStr">
-        <is>
-          <t>評判</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -3953,12 +3953,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
+          <t>小売り</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D94" s="12" t="inlineStr">
-        <is>
-          <t>小売り</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr">
@@ -3988,12 +3988,12 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
+          <t>寄付する</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>寄付する</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -4023,12 +4023,12 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
+          <t>納得させる</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D96" s="12" t="inlineStr">
-        <is>
-          <t>納得させる</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr">
@@ -4058,12 +4058,12 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
+          <t>分ける</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>分ける</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -4093,12 +4093,12 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
+          <t>罰金</t>
+        </is>
+      </c>
+      <c r="D98" s="12" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D98" s="12" t="inlineStr">
-        <is>
-          <t>罰金</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
@@ -4128,12 +4128,12 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
+          <t>尋ねる</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
           <t>動詞</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t>尋ねる</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -4163,12 +4163,12 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
+          <t>明確な・特定の</t>
+        </is>
+      </c>
+      <c r="D100" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D100" s="12" t="inlineStr">
-        <is>
-          <t>明確な・特定の</t>
         </is>
       </c>
       <c r="E100" s="13" t="inlineStr">
@@ -4198,12 +4198,12 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
+          <t>在庫</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
           <t>名詞</t>
-        </is>
-      </c>
-      <c r="D101" s="7" t="inlineStr">
-        <is>
-          <t>在庫</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -4233,12 +4233,12 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
+          <t>気が付いている</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D102" s="12" t="inlineStr">
-        <is>
-          <t>気が付いている</t>
         </is>
       </c>
       <c r="E102" s="13" t="inlineStr">
@@ -4268,12 +4268,12 @@
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
+          <t>大まかな</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t>大まかな</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -4303,12 +4303,12 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
+          <t>最大の</t>
+        </is>
+      </c>
+      <c r="D104" s="12" t="inlineStr">
+        <is>
           <t>形容詞</t>
-        </is>
-      </c>
-      <c r="D104" s="12" t="inlineStr">
-        <is>
-          <t>最大の</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Update quiz choices from A~J to 1~0 (including keyboard shortcut support)
</commit_message>
<xml_diff>
--- a/TOEIC_Words_401-500_100Quiz.xlsx
+++ b/TOEIC_Words_401-500_100Quiz.xlsx
@@ -4445,57 +4445,57 @@
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 A</t>
+          <t>選択肢 1</t>
         </is>
       </c>
       <c r="F5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 B</t>
+          <t>選択肢 2</t>
         </is>
       </c>
       <c r="G5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 C</t>
+          <t>選択肢 3</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 D</t>
+          <t>選択肢 4</t>
         </is>
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 E</t>
+          <t>選択肢 5</t>
         </is>
       </c>
       <c r="J5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 F</t>
+          <t>選択肢 6</t>
         </is>
       </c>
       <c r="K5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 G</t>
+          <t>選択肢 7</t>
         </is>
       </c>
       <c r="L5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 H</t>
+          <t>選択肢 8</t>
         </is>
       </c>
       <c r="M5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 I</t>
+          <t>選択肢 9</t>
         </is>
       </c>
       <c r="N5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 J</t>
+          <t>選択肢 0</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>あなたの回答 (A〜J)</t>
+          <t>あなたの回答 (1〜0)</t>
         </is>
       </c>
       <c r="P5" s="26" t="inlineStr">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="Q6" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R6" s="33" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="Q7" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R7" s="39" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="Q8" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R8" s="33" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="Q9" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R9" s="39" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="Q10" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R10" s="33" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="Q11" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R11" s="39" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="Q12" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R12" s="33" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="Q13" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R13" s="39" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="Q14" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R14" s="33" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="Q15" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R15" s="39" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="Q16" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R16" s="33" t="inlineStr">
@@ -5645,7 +5645,7 @@
       </c>
       <c r="Q17" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R17" s="39" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="Q18" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R18" s="33" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R19" s="39" t="inlineStr">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="Q20" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R20" s="33" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="Q21" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R21" s="39" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="Q22" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R22" s="33" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="Q23" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R23" s="39" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="Q24" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R24" s="33" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="Q25" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R25" s="39" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="Q26" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R26" s="33" t="inlineStr">
@@ -6595,7 +6595,7 @@
       </c>
       <c r="Q27" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R27" s="39" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="Q28" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R28" s="33" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="Q29" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R29" s="39" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="Q30" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R30" s="33" t="inlineStr">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="Q31" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R31" s="39" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="Q32" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R32" s="33" t="inlineStr">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="Q33" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R33" s="39" t="inlineStr">
@@ -7260,7 +7260,7 @@
       </c>
       <c r="Q34" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R34" s="33" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="Q35" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R35" s="39" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="Q36" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R36" s="33" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="Q37" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R37" s="39" t="inlineStr">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="Q38" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R38" s="33" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="Q39" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R39" s="39" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="Q40" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R40" s="33" t="inlineStr">
@@ -7925,7 +7925,7 @@
       </c>
       <c r="Q41" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R41" s="39" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="Q42" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R42" s="33" t="inlineStr">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="Q43" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R43" s="39" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="Q44" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R44" s="33" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="Q45" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R45" s="39" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="Q46" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R46" s="33" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="Q47" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R47" s="39" t="inlineStr">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="Q48" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R48" s="33" t="inlineStr">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="Q49" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R49" s="39" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="Q50" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R50" s="33" t="inlineStr">
@@ -8875,7 +8875,7 @@
       </c>
       <c r="Q51" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R51" s="39" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="Q52" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R52" s="33" t="inlineStr">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="Q53" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R53" s="39" t="inlineStr">
@@ -9160,7 +9160,7 @@
       </c>
       <c r="Q54" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R54" s="33" t="inlineStr">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="Q55" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R55" s="39" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="Q56" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R56" s="33" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="Q57" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R57" s="39" t="inlineStr">
@@ -9540,7 +9540,7 @@
       </c>
       <c r="Q58" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R58" s="33" t="inlineStr">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="Q59" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R59" s="39" t="inlineStr">
@@ -9730,7 +9730,7 @@
       </c>
       <c r="Q60" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R60" s="33" t="inlineStr">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="Q61" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R61" s="39" t="inlineStr">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="Q62" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R62" s="33" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="Q63" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R63" s="39" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="Q64" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R64" s="33" t="inlineStr">
@@ -10205,7 +10205,7 @@
       </c>
       <c r="Q65" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R65" s="39" t="inlineStr">
@@ -10300,7 +10300,7 @@
       </c>
       <c r="Q66" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R66" s="33" t="inlineStr">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="Q67" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R67" s="39" t="inlineStr">
@@ -10490,7 +10490,7 @@
       </c>
       <c r="Q68" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R68" s="33" t="inlineStr">
@@ -10585,7 +10585,7 @@
       </c>
       <c r="Q69" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R69" s="39" t="inlineStr">
@@ -10680,7 +10680,7 @@
       </c>
       <c r="Q70" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R70" s="33" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="Q71" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R71" s="39" t="inlineStr">
@@ -10870,7 +10870,7 @@
       </c>
       <c r="Q72" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R72" s="33" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="Q73" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R73" s="39" t="inlineStr">
@@ -11060,7 +11060,7 @@
       </c>
       <c r="Q74" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R74" s="33" t="inlineStr">
@@ -11155,7 +11155,7 @@
       </c>
       <c r="Q75" s="38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R75" s="39" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="Q76" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R76" s="33" t="inlineStr">
@@ -11345,7 +11345,7 @@
       </c>
       <c r="Q77" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R77" s="39" t="inlineStr">
@@ -11440,7 +11440,7 @@
       </c>
       <c r="Q78" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R78" s="33" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="Q79" s="38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R79" s="39" t="inlineStr">
@@ -11630,7 +11630,7 @@
       </c>
       <c r="Q80" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R80" s="33" t="inlineStr">
@@ -11725,7 +11725,7 @@
       </c>
       <c r="Q81" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R81" s="39" t="inlineStr">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="Q82" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R82" s="33" t="inlineStr">
@@ -11915,7 +11915,7 @@
       </c>
       <c r="Q83" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R83" s="39" t="inlineStr">
@@ -12010,7 +12010,7 @@
       </c>
       <c r="Q84" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R84" s="33" t="inlineStr">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="Q85" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R85" s="39" t="inlineStr">
@@ -12200,7 +12200,7 @@
       </c>
       <c r="Q86" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R86" s="33" t="inlineStr">
@@ -12295,7 +12295,7 @@
       </c>
       <c r="Q87" s="38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R87" s="39" t="inlineStr">
@@ -12390,7 +12390,7 @@
       </c>
       <c r="Q88" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R88" s="33" t="inlineStr">
@@ -12485,7 +12485,7 @@
       </c>
       <c r="Q89" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R89" s="39" t="inlineStr">
@@ -12580,7 +12580,7 @@
       </c>
       <c r="Q90" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R90" s="33" t="inlineStr">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="Q91" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R91" s="39" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="Q92" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R92" s="33" t="inlineStr">
@@ -12865,7 +12865,7 @@
       </c>
       <c r="Q93" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R93" s="39" t="inlineStr">
@@ -12960,7 +12960,7 @@
       </c>
       <c r="Q94" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R94" s="33" t="inlineStr">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="Q95" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R95" s="39" t="inlineStr">
@@ -13150,7 +13150,7 @@
       </c>
       <c r="Q96" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R96" s="33" t="inlineStr">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="Q97" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R97" s="39" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="Q98" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R98" s="33" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="Q99" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R99" s="39" t="inlineStr">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="Q100" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R100" s="33" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="Q101" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R101" s="39" t="inlineStr">
@@ -13720,7 +13720,7 @@
       </c>
       <c r="Q102" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R102" s="33" t="inlineStr">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="Q103" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R103" s="39" t="inlineStr">
@@ -13910,7 +13910,7 @@
       </c>
       <c r="Q104" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R104" s="33" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="Q105" s="38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R105" s="39" t="inlineStr">
@@ -14046,8 +14046,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="O6:O105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力エラー" error="AからJの英字を選択してください。" promptTitle="回答の選択" prompt="選択肢(A〜J)を選んでください" type="list">
-      <formula1>"A,B,C,D,E,F,G,H,I,J"</formula1>
+    <dataValidation sqref="O6:O105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力エラー" error="1から0の数字を選択してください。" promptTitle="回答の選択" prompt="選択肢(1〜0)を選んでください" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,0"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14162,57 +14162,57 @@
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 A</t>
+          <t>選択肢 1</t>
         </is>
       </c>
       <c r="F5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 B</t>
+          <t>選択肢 2</t>
         </is>
       </c>
       <c r="G5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 C</t>
+          <t>選択肢 3</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 D</t>
+          <t>選択肢 4</t>
         </is>
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 E</t>
+          <t>選択肢 5</t>
         </is>
       </c>
       <c r="J5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 F</t>
+          <t>選択肢 6</t>
         </is>
       </c>
       <c r="K5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 G</t>
+          <t>選択肢 7</t>
         </is>
       </c>
       <c r="L5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 H</t>
+          <t>選択肢 8</t>
         </is>
       </c>
       <c r="M5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 I</t>
+          <t>選択肢 9</t>
         </is>
       </c>
       <c r="N5" s="24" t="inlineStr">
         <is>
-          <t>選択肢 J</t>
+          <t>選択肢 0</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>あなたの回答 (A〜J)</t>
+          <t>あなたの回答 (1〜0)</t>
         </is>
       </c>
       <c r="P5" s="26" t="inlineStr">
@@ -14317,7 +14317,7 @@
       </c>
       <c r="Q6" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R6" s="33" t="inlineStr">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="Q7" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R7" s="39" t="inlineStr">
@@ -14507,7 +14507,7 @@
       </c>
       <c r="Q8" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R8" s="33" t="inlineStr">
@@ -14602,7 +14602,7 @@
       </c>
       <c r="Q9" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R9" s="39" t="inlineStr">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="Q10" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R10" s="33" t="inlineStr">
@@ -14792,7 +14792,7 @@
       </c>
       <c r="Q11" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R11" s="39" t="inlineStr">
@@ -14887,7 +14887,7 @@
       </c>
       <c r="Q12" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R12" s="33" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="Q13" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R13" s="39" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="Q14" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R14" s="33" t="inlineStr">
@@ -15172,7 +15172,7 @@
       </c>
       <c r="Q15" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R15" s="39" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="Q16" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R16" s="33" t="inlineStr">
@@ -15362,7 +15362,7 @@
       </c>
       <c r="Q17" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R17" s="39" t="inlineStr">
@@ -15457,7 +15457,7 @@
       </c>
       <c r="Q18" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R18" s="33" t="inlineStr">
@@ -15552,7 +15552,7 @@
       </c>
       <c r="Q19" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R19" s="39" t="inlineStr">
@@ -15647,7 +15647,7 @@
       </c>
       <c r="Q20" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R20" s="33" t="inlineStr">
@@ -15742,7 +15742,7 @@
       </c>
       <c r="Q21" s="38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R21" s="39" t="inlineStr">
@@ -15837,7 +15837,7 @@
       </c>
       <c r="Q22" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R22" s="33" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="Q23" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R23" s="39" t="inlineStr">
@@ -16027,7 +16027,7 @@
       </c>
       <c r="Q24" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R24" s="33" t="inlineStr">
@@ -16122,7 +16122,7 @@
       </c>
       <c r="Q25" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R25" s="39" t="inlineStr">
@@ -16217,7 +16217,7 @@
       </c>
       <c r="Q26" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R26" s="33" t="inlineStr">
@@ -16312,7 +16312,7 @@
       </c>
       <c r="Q27" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R27" s="39" t="inlineStr">
@@ -16407,7 +16407,7 @@
       </c>
       <c r="Q28" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R28" s="33" t="inlineStr">
@@ -16502,7 +16502,7 @@
       </c>
       <c r="Q29" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R29" s="39" t="inlineStr">
@@ -16597,7 +16597,7 @@
       </c>
       <c r="Q30" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R30" s="33" t="inlineStr">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="Q31" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R31" s="39" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="Q32" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R32" s="33" t="inlineStr">
@@ -16882,7 +16882,7 @@
       </c>
       <c r="Q33" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R33" s="39" t="inlineStr">
@@ -16977,7 +16977,7 @@
       </c>
       <c r="Q34" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R34" s="33" t="inlineStr">
@@ -17072,7 +17072,7 @@
       </c>
       <c r="Q35" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R35" s="39" t="inlineStr">
@@ -17167,7 +17167,7 @@
       </c>
       <c r="Q36" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R36" s="33" t="inlineStr">
@@ -17262,7 +17262,7 @@
       </c>
       <c r="Q37" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R37" s="39" t="inlineStr">
@@ -17357,7 +17357,7 @@
       </c>
       <c r="Q38" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R38" s="33" t="inlineStr">
@@ -17452,7 +17452,7 @@
       </c>
       <c r="Q39" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R39" s="39" t="inlineStr">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="Q40" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R40" s="33" t="inlineStr">
@@ -17642,7 +17642,7 @@
       </c>
       <c r="Q41" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R41" s="39" t="inlineStr">
@@ -17737,7 +17737,7 @@
       </c>
       <c r="Q42" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R42" s="33" t="inlineStr">
@@ -17832,7 +17832,7 @@
       </c>
       <c r="Q43" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R43" s="39" t="inlineStr">
@@ -17927,7 +17927,7 @@
       </c>
       <c r="Q44" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R44" s="33" t="inlineStr">
@@ -18022,7 +18022,7 @@
       </c>
       <c r="Q45" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R45" s="39" t="inlineStr">
@@ -18117,7 +18117,7 @@
       </c>
       <c r="Q46" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R46" s="33" t="inlineStr">
@@ -18212,7 +18212,7 @@
       </c>
       <c r="Q47" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R47" s="39" t="inlineStr">
@@ -18307,7 +18307,7 @@
       </c>
       <c r="Q48" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R48" s="33" t="inlineStr">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="Q49" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R49" s="39" t="inlineStr">
@@ -18497,7 +18497,7 @@
       </c>
       <c r="Q50" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R50" s="33" t="inlineStr">
@@ -18592,7 +18592,7 @@
       </c>
       <c r="Q51" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R51" s="39" t="inlineStr">
@@ -18687,7 +18687,7 @@
       </c>
       <c r="Q52" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R52" s="33" t="inlineStr">
@@ -18782,7 +18782,7 @@
       </c>
       <c r="Q53" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R53" s="39" t="inlineStr">
@@ -18877,7 +18877,7 @@
       </c>
       <c r="Q54" s="32" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R54" s="33" t="inlineStr">
@@ -18972,7 +18972,7 @@
       </c>
       <c r="Q55" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R55" s="39" t="inlineStr">
@@ -19067,7 +19067,7 @@
       </c>
       <c r="Q56" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R56" s="33" t="inlineStr">
@@ -19162,7 +19162,7 @@
       </c>
       <c r="Q57" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R57" s="39" t="inlineStr">
@@ -19257,7 +19257,7 @@
       </c>
       <c r="Q58" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R58" s="33" t="inlineStr">
@@ -19352,7 +19352,7 @@
       </c>
       <c r="Q59" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R59" s="39" t="inlineStr">
@@ -19447,7 +19447,7 @@
       </c>
       <c r="Q60" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R60" s="33" t="inlineStr">
@@ -19542,7 +19542,7 @@
       </c>
       <c r="Q61" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R61" s="39" t="inlineStr">
@@ -19637,7 +19637,7 @@
       </c>
       <c r="Q62" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R62" s="33" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="Q63" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R63" s="39" t="inlineStr">
@@ -19827,7 +19827,7 @@
       </c>
       <c r="Q64" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R64" s="33" t="inlineStr">
@@ -19922,7 +19922,7 @@
       </c>
       <c r="Q65" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R65" s="39" t="inlineStr">
@@ -20017,7 +20017,7 @@
       </c>
       <c r="Q66" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R66" s="33" t="inlineStr">
@@ -20112,7 +20112,7 @@
       </c>
       <c r="Q67" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R67" s="39" t="inlineStr">
@@ -20207,7 +20207,7 @@
       </c>
       <c r="Q68" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R68" s="33" t="inlineStr">
@@ -20302,7 +20302,7 @@
       </c>
       <c r="Q69" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R69" s="39" t="inlineStr">
@@ -20397,7 +20397,7 @@
       </c>
       <c r="Q70" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R70" s="33" t="inlineStr">
@@ -20492,7 +20492,7 @@
       </c>
       <c r="Q71" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R71" s="39" t="inlineStr">
@@ -20587,7 +20587,7 @@
       </c>
       <c r="Q72" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R72" s="33" t="inlineStr">
@@ -20682,7 +20682,7 @@
       </c>
       <c r="Q73" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R73" s="39" t="inlineStr">
@@ -20777,7 +20777,7 @@
       </c>
       <c r="Q74" s="32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R74" s="33" t="inlineStr">
@@ -20872,7 +20872,7 @@
       </c>
       <c r="Q75" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R75" s="39" t="inlineStr">
@@ -20967,7 +20967,7 @@
       </c>
       <c r="Q76" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R76" s="33" t="inlineStr">
@@ -21062,7 +21062,7 @@
       </c>
       <c r="Q77" s="38" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R77" s="39" t="inlineStr">
@@ -21157,7 +21157,7 @@
       </c>
       <c r="Q78" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R78" s="33" t="inlineStr">
@@ -21252,7 +21252,7 @@
       </c>
       <c r="Q79" s="38" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R79" s="39" t="inlineStr">
@@ -21347,7 +21347,7 @@
       </c>
       <c r="Q80" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R80" s="33" t="inlineStr">
@@ -21442,7 +21442,7 @@
       </c>
       <c r="Q81" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R81" s="39" t="inlineStr">
@@ -21537,7 +21537,7 @@
       </c>
       <c r="Q82" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R82" s="33" t="inlineStr">
@@ -21632,7 +21632,7 @@
       </c>
       <c r="Q83" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R83" s="39" t="inlineStr">
@@ -21727,7 +21727,7 @@
       </c>
       <c r="Q84" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R84" s="33" t="inlineStr">
@@ -21822,7 +21822,7 @@
       </c>
       <c r="Q85" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R85" s="39" t="inlineStr">
@@ -21917,7 +21917,7 @@
       </c>
       <c r="Q86" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R86" s="33" t="inlineStr">
@@ -22012,7 +22012,7 @@
       </c>
       <c r="Q87" s="38" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R87" s="39" t="inlineStr">
@@ -22107,7 +22107,7 @@
       </c>
       <c r="Q88" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R88" s="33" t="inlineStr">
@@ -22202,7 +22202,7 @@
       </c>
       <c r="Q89" s="38" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R89" s="39" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="Q90" s="32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R90" s="33" t="inlineStr">
@@ -22392,7 +22392,7 @@
       </c>
       <c r="Q91" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R91" s="39" t="inlineStr">
@@ -22487,7 +22487,7 @@
       </c>
       <c r="Q92" s="32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R92" s="33" t="inlineStr">
@@ -22582,7 +22582,7 @@
       </c>
       <c r="Q93" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R93" s="39" t="inlineStr">
@@ -22677,7 +22677,7 @@
       </c>
       <c r="Q94" s="32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R94" s="33" t="inlineStr">
@@ -22772,7 +22772,7 @@
       </c>
       <c r="Q95" s="38" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R95" s="39" t="inlineStr">
@@ -22867,7 +22867,7 @@
       </c>
       <c r="Q96" s="32" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R96" s="33" t="inlineStr">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="Q97" s="38" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R97" s="39" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="Q98" s="32" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R98" s="33" t="inlineStr">
@@ -23152,7 +23152,7 @@
       </c>
       <c r="Q99" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R99" s="39" t="inlineStr">
@@ -23247,7 +23247,7 @@
       </c>
       <c r="Q100" s="32" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R100" s="33" t="inlineStr">
@@ -23342,7 +23342,7 @@
       </c>
       <c r="Q101" s="38" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R101" s="39" t="inlineStr">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="Q102" s="32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R102" s="33" t="inlineStr">
@@ -23532,7 +23532,7 @@
       </c>
       <c r="Q103" s="38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R103" s="39" t="inlineStr">
@@ -23627,7 +23627,7 @@
       </c>
       <c r="Q104" s="32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R104" s="33" t="inlineStr">
@@ -23722,7 +23722,7 @@
       </c>
       <c r="Q105" s="38" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R105" s="39" t="inlineStr">
@@ -23763,8 +23763,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="O6:O105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力エラー" error="AからJの英字を選択してください。" promptTitle="回答の選択" prompt="選択肢(A〜J)を選んでください" type="list">
-      <formula1>"A,B,C,D,E,F,G,H,I,J"</formula1>
+    <dataValidation sqref="O6:O105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力エラー" error="1から0の数字を選択してください。" promptTitle="回答の選択" prompt="選択肢(1〜0)を選んでください" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,0"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>